<commit_message>
Sincronización automática: data/datos.xlsx, public/galeria/indumentaria.jpeg, public/galeria/cosam.jpeg
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -22,174 +22,174 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="760" uniqueCount="241">
   <si>
+    <t>cargo</t>
+  </si>
+  <si>
+    <t>anio</t>
+  </si>
+  <si>
     <t>nombre</t>
   </si>
   <si>
-    <t>anio</t>
-  </si>
-  <si>
     <t>apodo</t>
   </si>
   <si>
-    <t>cargo</t>
+    <t>fundacion</t>
+  </si>
+  <si>
+    <t>descripcion</t>
+  </si>
+  <si>
+    <t>foto</t>
+  </si>
+  <si>
+    <t>imagen</t>
+  </si>
+  <si>
+    <t>comuna</t>
+  </si>
+  <si>
+    <t>region</t>
+  </si>
+  <si>
+    <t>colores</t>
+  </si>
+  <si>
+    <t>Chocolo</t>
+  </si>
+  <si>
+    <t>estadio</t>
+  </si>
+  <si>
+    <t>El perro Chocolo es la mascota oficial del club. Acompaña al plantel en cada partido de local y anima a la hinchada desde la tribuna.</t>
+  </si>
+  <si>
+    <t>resumen</t>
+  </si>
+  <si>
+    <t>Presidente</t>
+  </si>
+  <si>
+    <t>/mascota/chocolo.jpeg</t>
+  </si>
+  <si>
+    <t>instagram</t>
+  </si>
+  <si>
+    <t>Feliciciano Barra</t>
   </si>
   <si>
     <t>titulo</t>
   </si>
   <si>
-    <t>fundacion</t>
+    <t>/directiva/feliciano-barra.jpeg</t>
+  </si>
+  <si>
+    <t>facebook</t>
   </si>
   <si>
     <t>texto</t>
   </si>
   <si>
-    <t>comuna</t>
-  </si>
-  <si>
-    <t>foto</t>
-  </si>
-  <si>
-    <t>region</t>
+    <t>Secretario</t>
+  </si>
+  <si>
+    <t>Daniel Muñoz</t>
+  </si>
+  <si>
+    <t>whatsapp</t>
   </si>
   <si>
     <t>1961</t>
   </si>
   <si>
-    <t>Presidente</t>
+    <t>/directiva/daniel-munoz.jpeg</t>
   </si>
   <si>
     <t>Fundación oficial del club</t>
   </si>
   <si>
-    <t>Feliciciano Barra</t>
-  </si>
-  <si>
-    <t>colores</t>
-  </si>
-  <si>
-    <t>/directiva/feliciano-barra.jpeg</t>
-  </si>
-  <si>
-    <t>estadio</t>
+    <t>Tesorero</t>
   </si>
   <si>
     <t>El 5 de noviembre de 1961, en medio de las masivas tomas de terreno de la zona sur de Santiago, un grupo de familias recién asentadas decide organizar un espacio de esparcimiento. Lo que comenzó con arcos de madera y una pelota de trapo en terrenos de tierra se convirtió en el nacimiento formal de la institución, uniendo a la comunidad a través del fútbol.</t>
   </si>
   <si>
-    <t>Secretario</t>
-  </si>
-  <si>
-    <t>Daniel Muñoz</t>
-  </si>
-  <si>
-    <t>resumen</t>
+    <t>Carlos Flores</t>
+  </si>
+  <si>
+    <t>Club Deportivo Juventud San Rafael</t>
+  </si>
+  <si>
+    <t>J con U, La Juve</t>
   </si>
   <si>
     <t>1986</t>
   </si>
   <si>
-    <t>/directiva/daniel-munoz.jpeg</t>
+    <t>1er Director</t>
   </si>
   <si>
     <t>Obtención de la Personalidad Jurídica</t>
   </si>
   <si>
-    <t>instagram</t>
+    <t>José Zarate</t>
   </si>
   <si>
     <t>El 24 de junio de 1986, en una época de alta complejidad social y política en el país, los dirigentes del club logran formalizar la institución legalmente. Este paso no solo les permitió competir en ligas locales de manera oficial, sino también postular a proyectos vecinales para mejorar sus equipamientos y transformarse en un pilar de resistencia comunitaria.</t>
   </si>
   <si>
-    <t>Tesorero</t>
-  </si>
-  <si>
-    <t>Carlos Flores</t>
-  </si>
-  <si>
-    <t>facebook</t>
+    <t>Segundo Director</t>
+  </si>
+  <si>
+    <t>Héctor Armingol</t>
+  </si>
+  <si>
+    <t>Rey Don Felipe 1330, La Pintana</t>
   </si>
   <si>
     <t>2011</t>
   </si>
   <si>
+    <t>Metropolitana</t>
+  </si>
+  <si>
     <t>Celebración de los 50 años de historia</t>
   </si>
   <si>
-    <t>1er Director</t>
-  </si>
-  <si>
-    <t>whatsapp</t>
-  </si>
-  <si>
-    <t>José Zarate</t>
+    <t>Rojo, Azul, Blanco</t>
   </si>
   <si>
     <t>El club cumple medio siglo de vida consolidado como una de las instituciones más antiguas y respetadas de La Pintana. La celebración reunió a fundadores, antiguos jugadores y a las nuevas generaciones, reforzando la identidad del club como una escuela de vida que ha rescatado a cientos de jóvenes de la exclusión social.</t>
   </si>
   <si>
-    <t>Club Deportivo Juventud San Rafael</t>
-  </si>
-  <si>
-    <t>Segundo Director</t>
-  </si>
-  <si>
-    <t>J con U, La Juve</t>
-  </si>
-  <si>
-    <t>Héctor Armingol</t>
+    <t>Estadio Municipal de La Pintana, Complejo Deportivo Las Rosas, Estadio Rául del Canto</t>
   </si>
   <si>
     <t>2018</t>
   </si>
   <si>
+    <t>Fundado por un grupo de vecinos de San Rafael, el club nació como espacio de encuentro y hoy reúne a más de 300 jugadoras y jugadores en sus distintas series, desde Escuela de Fútbol hasta el plantel adulto.</t>
+  </si>
+  <si>
     <t>Inauguración de mejoras en el Complejo Deportivo San Rafael</t>
   </si>
   <si>
-    <t>Rey Don Felipe 1330, La Pintana</t>
-  </si>
-  <si>
-    <t>Metropolitana</t>
-  </si>
-  <si>
     <t>Gracias a la gestión comunitaria y el apoyo municipal, se materializan proyectos de luminarias y mejoras en la cancha del barrio. Esto permitió al club ampliar sus horarios de entrenamiento nocturnos, integrando de forma masiva series infantiles, juveniles y adultas en un entorno mucho más seguro y digno.</t>
   </si>
   <si>
-    <t>Rojo, Azul, Blanco</t>
-  </si>
-  <si>
-    <t>descripcion</t>
-  </si>
-  <si>
-    <t>Estadio Municipal de La Pintana, Complejo Deportivo Las Rosas, Estadio Rául del Canto</t>
+    <t>https://instagram.com/club_juventudsanrafael</t>
   </si>
   <si>
     <t>2024</t>
   </si>
   <si>
-    <t>imagen</t>
-  </si>
-  <si>
-    <t>Fundado por un grupo de vecinos de San Rafael, el club nació como espacio de encuentro y hoy reúne a más de 300 jugadoras y jugadores en sus distintas series, desde Escuela de Fútbol hasta el plantel adulto.</t>
-  </si>
-  <si>
     <t>Campaña por la Paz y Fútbol Formativo</t>
   </si>
   <si>
-    <t>https://instagram.com/club_juventudsanrafael</t>
-  </si>
-  <si>
     <t>Lanzamiento oficial de la campaña "No más violencia en las canchas". Ante el aumento de la delincuencia y los roces en el fútbol amateur de Santiago, Juventud San Rafael se convierte en un referente comunal al liderar iniciativas de convivencia escolar y deportiva. El club reafirma su rol como "escuela formativa", priorizando los valores, la disciplina y la vida sana por sobre los resultados en el marcador.</t>
   </si>
   <si>
-    <t>Chocolo</t>
-  </si>
-  <si>
-    <t>El perro Chocolo es la mascota oficial del club. Acompaña al plantel en cada partido de local y anima a la hinchada desde la tribuna.</t>
-  </si>
-  <si>
-    <t>/mascota/chocolo.jpeg</t>
-  </si>
-  <si>
     <t>https://www.facebook.com/clubjuventudsnrafael</t>
   </si>
   <si>
@@ -367,70 +367,79 @@
     <t>Sergio Moscoso</t>
   </si>
   <si>
+    <t>liga</t>
+  </si>
+  <si>
     <t>David Ceballo</t>
   </si>
   <si>
+    <t>actualizado</t>
+  </si>
+  <si>
+    <t>pos</t>
+  </si>
+  <si>
     <t>Smiljan Becerra</t>
   </si>
   <si>
+    <t>equipo</t>
+  </si>
+  <si>
+    <t>pj</t>
+  </si>
+  <si>
     <t>Cristian Lara</t>
   </si>
   <si>
-    <t>liga</t>
-  </si>
-  <si>
-    <t>actualizado</t>
+    <t>pg</t>
+  </si>
+  <si>
+    <t>pe</t>
+  </si>
+  <si>
+    <t>pp</t>
+  </si>
+  <si>
+    <t>gf</t>
   </si>
   <si>
     <t>Marco Castillo</t>
   </si>
   <si>
-    <t>pos</t>
-  </si>
-  <si>
-    <t>equipo</t>
+    <t>gc</t>
+  </si>
+  <si>
+    <t>pts</t>
   </si>
   <si>
     <t>Ariel Bustamante</t>
   </si>
   <si>
-    <t>pj</t>
-  </si>
-  <si>
-    <t>pg</t>
+    <t>Santa Rosa Sur</t>
+  </si>
+  <si>
+    <t>2026-08-26</t>
+  </si>
+  <si>
+    <t>Juventud San Rafael</t>
   </si>
   <si>
     <t>Angelo Soto</t>
   </si>
   <si>
-    <t>pe</t>
-  </si>
-  <si>
     <t>Dean Castillo</t>
   </si>
   <si>
-    <t>pp</t>
-  </si>
-  <si>
-    <t>gf</t>
-  </si>
-  <si>
     <t>Victor Huera</t>
   </si>
   <si>
-    <t>gc</t>
-  </si>
-  <si>
-    <t>pts</t>
+    <t>Green Cross</t>
   </si>
   <si>
     <t>Emanuel Saavedra</t>
   </si>
   <si>
-    <t>Santa Rosa Sur</t>
-  </si>
-  <si>
-    <t>2026-08-26</t>
+    <t>Jorge Toro</t>
   </si>
   <si>
     <t>Delantero</t>
@@ -439,19 +448,19 @@
     <t>/jugadores/jonathan-ortega.jpeg</t>
   </si>
   <si>
-    <t>Juventud San Rafael</t>
-  </si>
-  <si>
     <t>Sebastián Fuentes</t>
   </si>
   <si>
     <t>/jugadores/sebastian-fuentes.jpeg</t>
   </si>
   <si>
+    <t>Juventud Santos</t>
+  </si>
+  <si>
     <t>/jugadores/alexis-alegria.jpeg</t>
   </si>
   <si>
-    <t>Green Cross</t>
+    <t>Santos Bilbao</t>
   </si>
   <si>
     <t>Emerson Castro</t>
@@ -460,28 +469,31 @@
     <t>Maximiliano Armijo</t>
   </si>
   <si>
-    <t>Jorge Toro</t>
+    <t>Huracán</t>
   </si>
   <si>
     <t>Erick Gonzalez</t>
   </si>
   <si>
+    <t>San Francisco</t>
+  </si>
+  <si>
     <t>Stiven Rodriguez</t>
   </si>
   <si>
-    <t>Juventud Santos</t>
-  </si>
-  <si>
     <t>Marcelo Palma</t>
   </si>
   <si>
+    <t>Atlético Español</t>
+  </si>
+  <si>
     <t>Hernan Herrera</t>
   </si>
   <si>
     <t>Jose Aleguy</t>
   </si>
   <si>
-    <t>Santos Bilbao</t>
+    <t>Juventud Nueva Estrella</t>
   </si>
   <si>
     <t>Cristian Silva</t>
@@ -490,9 +502,6 @@
     <t>Alvaro Vasquez</t>
   </si>
   <si>
-    <t>Huracán</t>
-  </si>
-  <si>
     <t>Arle Paredes</t>
   </si>
   <si>
@@ -502,9 +511,6 @@
     <t>Mauricio Vasquez</t>
   </si>
   <si>
-    <t>San Francisco</t>
-  </si>
-  <si>
     <t>Cristian Gonzalez</t>
   </si>
   <si>
@@ -514,9 +520,6 @@
     <t>Marco Uribe</t>
   </si>
   <si>
-    <t>Atlético Español</t>
-  </si>
-  <si>
     <t>Pablo Rubilar</t>
   </si>
   <si>
@@ -526,9 +529,6 @@
     <t>Rolando Rojas</t>
   </si>
   <si>
-    <t>Juventud Nueva Estrella</t>
-  </si>
-  <si>
     <t>Jesus Vasquez</t>
   </si>
   <si>
@@ -580,6 +580,9 @@
     <t>21:00</t>
   </si>
   <si>
+    <t>lugar</t>
+  </si>
+  <si>
     <t>Local</t>
   </si>
   <si>
@@ -589,12 +592,36 @@
     <t>No informado</t>
   </si>
   <si>
+    <t>Escuela de Fútbol</t>
+  </si>
+  <si>
     <t>2026-08-29</t>
   </si>
   <si>
+    <t>2026-09-01</t>
+  </si>
+  <si>
     <t>14:00</t>
   </si>
   <si>
+    <t>Sede social del club y Formulario de Contacto</t>
+  </si>
+  <si>
+    <t>Se invita a niños y niñas a particiar en la Escuela de Fútbol.</t>
+  </si>
+  <si>
+    <t>Aniversario N°65 del club</t>
+  </si>
+  <si>
+    <t>2026-11-05</t>
+  </si>
+  <si>
+    <t>Sede social del club</t>
+  </si>
+  <si>
+    <t>Celebramos un año más de historia con eventos deportivos para los niños y actividades extraprogramáticas para los adultos.</t>
+  </si>
+  <si>
     <t>14:50</t>
   </si>
   <si>
@@ -604,40 +631,13 @@
     <t>16:40</t>
   </si>
   <si>
-    <t>lugar</t>
-  </si>
-  <si>
     <t>17:50</t>
   </si>
   <si>
-    <t>Escuela de Fútbol</t>
-  </si>
-  <si>
-    <t>2026-09-01</t>
-  </si>
-  <si>
     <t>1 - 5</t>
   </si>
   <si>
-    <t>Sede social del club y Formulario de Contacto</t>
-  </si>
-  <si>
-    <t>Se invita a niños y niñas a particiar en la Escuela de Fútbol.</t>
-  </si>
-  <si>
     <t>19:00</t>
-  </si>
-  <si>
-    <t>Aniversario N°65 del club</t>
-  </si>
-  <si>
-    <t>2026-11-05</t>
-  </si>
-  <si>
-    <t>Sede social del club</t>
-  </si>
-  <si>
-    <t>Celebramos un año más de historia con eventos deportivos para los niños y actividades extraprogramáticas para los adultos.</t>
   </si>
   <si>
     <t>2 - 1</t>
@@ -1041,45 +1041,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="I1" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C2" s="1">
         <v>1961.0</v>
@@ -1088,19 +1088,19 @@
         <v>41</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>49</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>56</v>
@@ -2114,7 +2114,7 @@
         <v>215</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>216</v>
@@ -3315,65 +3315,65 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21"/>
@@ -4373,59 +4373,59 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21"/>
@@ -5425,24 +5425,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>54</v>
+        <v>13</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>55</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21"/>
@@ -6445,7 +6445,7 @@
         <v>58</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>59</v>
@@ -7572,13 +7572,13 @@
         <v>84</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>85</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
@@ -7787,7 +7787,7 @@
         <v>78</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>108</v>
@@ -7798,7 +7798,7 @@
         <v>78</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>108</v>
@@ -7809,7 +7809,7 @@
         <v>78</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>108</v>
@@ -7820,7 +7820,7 @@
         <v>78</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>108</v>
@@ -7831,7 +7831,7 @@
         <v>78</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>108</v>
@@ -7842,7 +7842,7 @@
         <v>78</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>108</v>
@@ -7853,7 +7853,7 @@
         <v>78</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>108</v>
@@ -7864,7 +7864,7 @@
         <v>78</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>108</v>
@@ -7875,7 +7875,7 @@
         <v>78</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>108</v>
@@ -7889,10 +7889,10 @@
         <v>82</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="27">
@@ -7900,13 +7900,13 @@
         <v>78</v>
       </c>
       <c r="C27" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="D27" s="1" t="s">
-        <v>137</v>
-      </c>
       <c r="E27" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="28">
@@ -7920,10 +7920,10 @@
         <v>70</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="29">
@@ -7931,10 +7931,10 @@
         <v>78</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="30">
@@ -7942,10 +7942,10 @@
         <v>78</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="31">
@@ -7967,7 +7967,7 @@
         <v>1.0</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>89</v>
@@ -7978,7 +7978,7 @@
         <v>80</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>94</v>
@@ -7989,7 +7989,7 @@
         <v>80</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>94</v>
@@ -8000,10 +8000,10 @@
         <v>80</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="36">
@@ -8011,10 +8011,10 @@
         <v>80</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="37">
@@ -8022,10 +8022,10 @@
         <v>80</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="38">
@@ -8033,10 +8033,10 @@
         <v>80</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="39">
@@ -8044,10 +8044,10 @@
         <v>80</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="40">
@@ -8055,10 +8055,10 @@
         <v>80</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="41">
@@ -8066,10 +8066,10 @@
         <v>80</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="42">
@@ -8077,10 +8077,10 @@
         <v>80</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="43">
@@ -8088,10 +8088,10 @@
         <v>80</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="44">
@@ -8099,10 +8099,10 @@
         <v>80</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="45">
@@ -8110,10 +8110,10 @@
         <v>80</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="46">
@@ -8121,10 +8121,10 @@
         <v>80</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="47">
@@ -8132,10 +8132,10 @@
         <v>80</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="48">
@@ -8143,10 +8143,10 @@
         <v>80</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="49">
@@ -8157,7 +8157,7 @@
         <v>169</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="50">
@@ -8168,7 +8168,7 @@
         <v>170</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="51">
@@ -8179,7 +8179,7 @@
         <v>171</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="52">
@@ -8190,7 +8190,7 @@
         <v>172</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="53">
@@ -8201,7 +8201,7 @@
         <v>173</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="54">
@@ -8212,7 +8212,7 @@
         <v>174</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="55">
@@ -8223,7 +8223,7 @@
         <v>175</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="56">
@@ -8234,7 +8234,7 @@
         <v>176</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="57"/>
@@ -9201,37 +9201,37 @@
         <v>83</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="2">
@@ -9239,16 +9239,16 @@
         <v>78</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D2" s="1">
         <v>1.0</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="F2" s="1">
         <v>0.0</v>
@@ -9277,16 +9277,16 @@
         <v>78</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D3" s="1">
         <v>2.0</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="F3" s="1">
         <v>0.0</v>
@@ -9315,16 +9315,16 @@
         <v>78</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D4" s="1">
         <v>3.0</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="F4" s="1">
         <v>0.0</v>
@@ -9353,16 +9353,16 @@
         <v>78</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D5" s="1">
         <v>4.0</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="F5" s="1">
         <v>0.0</v>
@@ -9391,16 +9391,16 @@
         <v>78</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D6" s="1">
         <v>5.0</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="F6" s="1">
         <v>0.0</v>
@@ -9429,16 +9429,16 @@
         <v>78</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D7" s="1">
         <v>6.0</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="F7" s="1">
         <v>0.0</v>
@@ -9467,16 +9467,16 @@
         <v>78</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D8" s="1">
         <v>7.0</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="F8" s="1">
         <v>0.0</v>
@@ -9505,16 +9505,16 @@
         <v>78</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D9" s="1">
         <v>8.0</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="F9" s="1">
         <v>0.0</v>
@@ -9543,16 +9543,16 @@
         <v>78</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D10" s="1">
         <v>9.0</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="F10" s="1">
         <v>0.0</v>
@@ -9581,16 +9581,16 @@
         <v>80</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D11" s="1">
         <v>1.0</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="F11" s="1">
         <v>0.0</v>
@@ -9619,16 +9619,16 @@
         <v>80</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D12" s="1">
         <v>2.0</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="F12" s="1">
         <v>0.0</v>
@@ -9657,16 +9657,16 @@
         <v>80</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D13" s="1">
         <v>3.0</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="F13" s="1">
         <v>0.0</v>
@@ -9695,16 +9695,16 @@
         <v>80</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D14" s="1">
         <v>4.0</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="F14" s="1">
         <v>0.0</v>
@@ -9733,16 +9733,16 @@
         <v>80</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D15" s="1">
         <v>5.0</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="F15" s="1">
         <v>0.0</v>
@@ -9771,16 +9771,16 @@
         <v>80</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D16" s="1">
         <v>6.0</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="F16" s="1">
         <v>0.0</v>
@@ -9809,16 +9809,16 @@
         <v>80</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D17" s="1">
         <v>7.0</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="F17" s="1">
         <v>0.0</v>
@@ -9847,16 +9847,16 @@
         <v>80</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D18" s="1">
         <v>8.0</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="F18" s="1">
         <v>0.0</v>
@@ -9885,16 +9885,16 @@
         <v>80</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D19" s="1">
         <v>9.0</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="F19" s="1">
         <v>0.0</v>
@@ -9923,16 +9923,16 @@
         <v>62</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D20" s="1">
         <v>1.0</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="F20" s="1">
         <v>0.0</v>
@@ -9961,16 +9961,16 @@
         <v>62</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D21" s="1">
         <v>2.0</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="F21" s="1">
         <v>0.0</v>
@@ -9999,16 +9999,16 @@
         <v>62</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D22" s="1">
         <v>3.0</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="F22" s="1">
         <v>0.0</v>
@@ -10037,16 +10037,16 @@
         <v>62</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D23" s="1">
         <v>4.0</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="F23" s="1">
         <v>0.0</v>
@@ -10075,16 +10075,16 @@
         <v>62</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D24" s="1">
         <v>5.0</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="F24" s="1">
         <v>0.0</v>
@@ -10113,16 +10113,16 @@
         <v>62</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D25" s="1">
         <v>6.0</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="F25" s="1">
         <v>0.0</v>
@@ -10151,16 +10151,16 @@
         <v>62</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D26" s="1">
         <v>7.0</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="F26" s="1">
         <v>0.0</v>
@@ -10189,16 +10189,16 @@
         <v>62</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D27" s="1">
         <v>8.0</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="F27" s="1">
         <v>0.0</v>
@@ -10227,16 +10227,16 @@
         <v>62</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D28" s="1">
         <v>9.0</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="F28" s="1">
         <v>0.0</v>
@@ -10265,16 +10265,16 @@
         <v>66</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D29" s="1">
         <v>1.0</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="F29" s="1">
         <v>0.0</v>
@@ -10303,16 +10303,16 @@
         <v>66</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D30" s="1">
         <v>2.0</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="F30" s="1">
         <v>0.0</v>
@@ -10341,16 +10341,16 @@
         <v>66</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D31" s="1">
         <v>3.0</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="F31" s="1">
         <v>0.0</v>
@@ -10379,16 +10379,16 @@
         <v>66</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D32" s="1">
         <v>4.0</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="F32" s="1">
         <v>0.0</v>
@@ -10417,16 +10417,16 @@
         <v>66</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D33" s="1">
         <v>5.0</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="F33" s="1">
         <v>0.0</v>
@@ -10455,16 +10455,16 @@
         <v>66</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D34" s="1">
         <v>6.0</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="F34" s="1">
         <v>0.0</v>
@@ -10493,16 +10493,16 @@
         <v>66</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D35" s="1">
         <v>7.0</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="F35" s="1">
         <v>0.0</v>
@@ -10531,16 +10531,16 @@
         <v>66</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D36" s="1">
         <v>8.0</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="F36" s="1">
         <v>0.0</v>
@@ -10569,16 +10569,16 @@
         <v>66</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D37" s="1">
         <v>9.0</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="F37" s="1">
         <v>0.0</v>
@@ -10607,16 +10607,16 @@
         <v>68</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D38" s="1">
         <v>1.0</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="F38" s="1">
         <v>0.0</v>
@@ -10645,16 +10645,16 @@
         <v>68</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D39" s="1">
         <v>2.0</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="F39" s="1">
         <v>0.0</v>
@@ -10683,16 +10683,16 @@
         <v>68</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D40" s="1">
         <v>3.0</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="F40" s="1">
         <v>0.0</v>
@@ -10721,16 +10721,16 @@
         <v>68</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D41" s="1">
         <v>4.0</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="F41" s="1">
         <v>0.0</v>
@@ -10759,16 +10759,16 @@
         <v>68</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D42" s="1">
         <v>5.0</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="F42" s="1">
         <v>0.0</v>
@@ -10797,16 +10797,16 @@
         <v>68</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D43" s="1">
         <v>6.0</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="F43" s="1">
         <v>0.0</v>
@@ -10835,16 +10835,16 @@
         <v>68</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D44" s="1">
         <v>7.0</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="F44" s="1">
         <v>0.0</v>
@@ -10873,16 +10873,16 @@
         <v>68</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D45" s="1">
         <v>8.0</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="F45" s="1">
         <v>0.0</v>
@@ -10911,16 +10911,16 @@
         <v>68</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D46" s="1">
         <v>9.0</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="F46" s="1">
         <v>0.0</v>
@@ -10949,16 +10949,16 @@
         <v>71</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D47" s="1">
         <v>1.0</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="F47" s="1">
         <v>0.0</v>
@@ -10987,16 +10987,16 @@
         <v>71</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D48" s="1">
         <v>2.0</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="F48" s="1">
         <v>0.0</v>
@@ -11025,16 +11025,16 @@
         <v>71</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D49" s="1">
         <v>3.0</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="F49" s="1">
         <v>0.0</v>
@@ -11063,16 +11063,16 @@
         <v>71</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D50" s="1">
         <v>4.0</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="F50" s="1">
         <v>0.0</v>
@@ -11101,16 +11101,16 @@
         <v>71</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D51" s="1">
         <v>5.0</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="F51" s="1">
         <v>0.0</v>
@@ -11139,16 +11139,16 @@
         <v>71</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D52" s="1">
         <v>6.0</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="F52" s="1">
         <v>0.0</v>
@@ -11177,16 +11177,16 @@
         <v>71</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D53" s="1">
         <v>7.0</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="F53" s="1">
         <v>0.0</v>
@@ -11215,16 +11215,16 @@
         <v>71</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D54" s="1">
         <v>8.0</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="F54" s="1">
         <v>0.0</v>
@@ -11253,16 +11253,16 @@
         <v>71</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D55" s="1">
         <v>9.0</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="F55" s="1">
         <v>0.0</v>
@@ -11291,16 +11291,16 @@
         <v>74</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D56" s="1">
         <v>1.0</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="F56" s="1">
         <v>0.0</v>
@@ -11329,16 +11329,16 @@
         <v>74</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D57" s="1">
         <v>2.0</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="F57" s="1">
         <v>0.0</v>
@@ -11367,16 +11367,16 @@
         <v>74</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D58" s="1">
         <v>3.0</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="F58" s="1">
         <v>0.0</v>
@@ -11405,16 +11405,16 @@
         <v>74</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D59" s="1">
         <v>4.0</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="F59" s="1">
         <v>0.0</v>
@@ -11443,16 +11443,16 @@
         <v>74</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D60" s="1">
         <v>5.0</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="F60" s="1">
         <v>0.0</v>
@@ -11481,16 +11481,16 @@
         <v>74</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D61" s="1">
         <v>6.0</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="F61" s="1">
         <v>0.0</v>
@@ -11519,16 +11519,16 @@
         <v>74</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D62" s="1">
         <v>7.0</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="F62" s="1">
         <v>0.0</v>
@@ -11557,16 +11557,16 @@
         <v>74</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D63" s="1">
         <v>8.0</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="F63" s="1">
         <v>0.0</v>
@@ -11595,16 +11595,16 @@
         <v>74</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D64" s="1">
         <v>9.0</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="F64" s="1">
         <v>0.0</v>
@@ -11633,16 +11633,16 @@
         <v>76</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D65" s="1">
         <v>1.0</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="F65" s="1">
         <v>0.0</v>
@@ -11671,16 +11671,16 @@
         <v>76</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D66" s="1">
         <v>2.0</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="F66" s="1">
         <v>0.0</v>
@@ -11709,16 +11709,16 @@
         <v>76</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D67" s="1">
         <v>3.0</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="F67" s="1">
         <v>0.0</v>
@@ -11747,16 +11747,16 @@
         <v>76</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D68" s="1">
         <v>4.0</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="F68" s="1">
         <v>0.0</v>
@@ -11785,16 +11785,16 @@
         <v>76</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D69" s="1">
         <v>5.0</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="F69" s="1">
         <v>0.0</v>
@@ -11823,16 +11823,16 @@
         <v>76</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D70" s="1">
         <v>6.0</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="F70" s="1">
         <v>0.0</v>
@@ -11861,16 +11861,16 @@
         <v>76</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D71" s="1">
         <v>7.0</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="F71" s="1">
         <v>0.0</v>
@@ -11899,16 +11899,16 @@
         <v>76</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D72" s="1">
         <v>8.0</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="F72" s="1">
         <v>0.0</v>
@@ -11937,16 +11937,16 @@
         <v>76</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D73" s="1">
         <v>9.0</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="F73" s="1">
         <v>0.0</v>
@@ -12946,151 +12946,151 @@
         <v>81</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>67</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>69</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>72</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>75</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>79</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>206</v>
@@ -13098,7 +13098,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>207</v>
@@ -13107,13 +13107,13 @@
         <v>77</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>208</v>
@@ -13121,7 +13121,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>209</v>
@@ -13133,13 +13133,13 @@
         <v>211</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>211</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="11">
@@ -13153,10 +13153,10 @@
         <v>81</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>213</v>
@@ -13167,16 +13167,16 @@
         <v>214</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>213</v>
@@ -13187,16 +13187,16 @@
         <v>214</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>67</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>213</v>
@@ -13207,16 +13207,16 @@
         <v>214</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>69</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>213</v>
@@ -13227,16 +13227,16 @@
         <v>214</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>72</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>213</v>
@@ -13247,16 +13247,16 @@
         <v>214</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>75</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>213</v>
@@ -13267,16 +13267,16 @@
         <v>214</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>79</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>213</v>
@@ -13293,10 +13293,10 @@
         <v>77</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>213</v>
@@ -13316,7 +13316,7 @@
         <v>211</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>211</v>
@@ -14319,47 +14319,47 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>177</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
     </row>
     <row r="21"/>

</xml_diff>